<commit_message>
Cashiering FRS v3.2 and Product Maintenance FRS v1.2 rebuilt: the reinstatement setting named in words, insurer screens with business addresses; highlighted copies and workbooks rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_Inputs_BRD-02_Business_Unit_Requirements_Collection_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_Inputs_BRD-02_Business_Unit_Requirements_Collection_v1.0.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Documents and print formats'!$12:$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'E-mail wordings'!$A$12:$K$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'E-mail wordings'!$12:$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Messages to confirm'!$A$12:$K$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Messages to confirm'!$A$12:$K$162</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Messages to confirm'!$12:$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Schedules and timings'!$A$12:$K$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Schedules and timings'!$12:$12</definedName>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D24" s="12" t="n">
-        <v>131</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>131 items</t>
+          <t>149 items</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F7" s="22" t="n">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="G7" s="22">
         <f>COUNTIF('Messages to confirm'!K:K,"Open")</f>
@@ -13259,7 +13259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K144"/>
+  <dimension ref="A1:K162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14111,12 +14111,12 @@
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>M-020</t>
+          <t>M-049</t>
         </is>
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
+          <t>AR and OR Forms and printing (SCR-OP-69, SCR-OP-18)</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
@@ -14131,7 +14131,7 @@
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A reclass or transfer moves the whole balance" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The effective date must be today or a later date" (type Error).</t>
         </is>
       </c>
       <c r="F22" s="22" t="inlineStr">
@@ -14164,12 +14164,12 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>M-021</t>
+          <t>M-050</t>
         </is>
       </c>
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
+          <t>AR and OR Forms and printing (SCR-OP-69, SCR-OP-18)</t>
         </is>
       </c>
       <c r="C23" s="24" t="inlineStr">
@@ -14184,7 +14184,7 @@
       </c>
       <c r="E23" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Check number is required for a check payment" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Select the AR form or the OR form" (type Error).</t>
         </is>
       </c>
       <c r="F23" s="24" t="inlineStr">
@@ -14217,12 +14217,12 @@
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>M-022</t>
+          <t>M-051</t>
         </is>
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
+          <t>AR and OR Forms and printing (SCR-OP-69, SCR-OP-18)</t>
         </is>
       </c>
       <c r="C24" s="22" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="E24" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an ARN, invoice, policy or PN number to preview the application." (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the reason for the rejection" (type Error).</t>
         </is>
       </c>
       <c r="F24" s="22" t="inlineStr">
@@ -14270,7 +14270,7 @@
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>M-023</t>
+          <t>M-053</t>
         </is>
       </c>
       <c r="B25" s="24" t="inlineStr">
@@ -14290,7 +14290,7 @@
       </c>
       <c r="E25" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A reclass or transfer moves the whole balance" (type Validation).</t>
         </is>
       </c>
       <c r="F25" s="24" t="inlineStr">
@@ -14323,7 +14323,7 @@
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>M-024</t>
+          <t>M-054</t>
         </is>
       </c>
       <c r="B26" s="22" t="inlineStr">
@@ -14343,7 +14343,7 @@
       </c>
       <c r="E26" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most &lt;balance&gt;" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Check number is required for a check payment" (type Validation).</t>
         </is>
       </c>
       <c r="F26" s="22" t="inlineStr">
@@ -14376,7 +14376,7 @@
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>M-025</t>
+          <t>M-055</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most &lt;receipt amount&gt;" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an ARN, invoice, policy or PN number to preview the application." (type Validation).</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
@@ -14429,7 +14429,7 @@
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
         <is>
-          <t>M-026</t>
+          <t>M-056</t>
         </is>
       </c>
       <c r="B28" s="22" t="inlineStr">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="E28" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter at least one reference, or the payor code for an unmatched payment" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero" (type Validation).</t>
         </is>
       </c>
       <c r="F28" s="22" t="inlineStr">
@@ -14482,7 +14482,7 @@
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>M-027</t>
+          <t>M-057</t>
         </is>
       </c>
       <c r="B29" s="24" t="inlineStr">
@@ -14502,7 +14502,7 @@
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Payor name is required" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most &lt;balance&gt;" (type Validation).</t>
         </is>
       </c>
       <c r="F29" s="24" t="inlineStr">
@@ -14535,7 +14535,7 @@
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
         <is>
-          <t>M-028</t>
+          <t>M-058</t>
         </is>
       </c>
       <c r="B30" s="22" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="E30" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Select a reason" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most &lt;receipt amount&gt;" (type Validation).</t>
         </is>
       </c>
       <c r="F30" s="22" t="inlineStr">
@@ -14588,7 +14588,7 @@
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>M-029</t>
+          <t>M-059</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The reference belongs to a cancelled invoice: the payment goes to unapplied collections." (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter at least one reference, or the payor code for an unmatched payment" (type Validation).</t>
         </is>
       </c>
       <c r="F31" s="24" t="inlineStr">
@@ -14641,7 +14641,7 @@
     <row r="32">
       <c r="A32" s="22" t="inlineStr">
         <is>
-          <t>M-030</t>
+          <t>M-060</t>
         </is>
       </c>
       <c r="B32" s="22" t="inlineStr">
@@ -14661,7 +14661,7 @@
       </c>
       <c r="E32" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Application &lt;id&gt; is already reversed" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Payor name is required" (type Validation).</t>
         </is>
       </c>
       <c r="F32" s="22" t="inlineStr">
@@ -14694,7 +14694,7 @@
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>M-031</t>
+          <t>M-061</t>
         </is>
       </c>
       <c r="B33" s="24" t="inlineStr">
@@ -14714,7 +14714,7 @@
       </c>
       <c r="E33" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A non-premium AR needs the paying insurer's code" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Select a reason" (type Validation).</t>
         </is>
       </c>
       <c r="F33" s="24" t="inlineStr">
@@ -14747,7 +14747,7 @@
     <row r="34">
       <c r="A34" s="22" t="inlineStr">
         <is>
-          <t>M-032</t>
+          <t>M-062</t>
         </is>
       </c>
       <c r="B34" s="22" t="inlineStr">
@@ -14767,7 +14767,7 @@
       </c>
       <c r="E34" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Official receipts are issued by Head Office only" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The reference belongs to a cancelled invoice: the payment goes to unapplied collections." (type Validation).</t>
         </is>
       </c>
       <c r="F34" s="22" t="inlineStr">
@@ -14800,7 +14800,7 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>M-033</t>
+          <t>M-063</t>
         </is>
       </c>
       <c r="B35" s="24" t="inlineStr">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="E35" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "An official receipt needs a line" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Application &lt;id&gt; is already reversed" (type Error).</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
@@ -14853,7 +14853,7 @@
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>M-034</t>
+          <t>M-064</t>
         </is>
       </c>
       <c r="B36" s="22" t="inlineStr">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="E36" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A receipt needs an amount above zero" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A non-premium AR needs the paying insurer's code" (type Error).</t>
         </is>
       </c>
       <c r="F36" s="22" t="inlineStr">
@@ -14906,12 +14906,12 @@
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>M-035</t>
+          <t>M-065</t>
         </is>
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
+          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -14926,7 +14926,7 @@
       </c>
       <c r="E37" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;receipt no&gt; issued" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Official receipts are issued by Head Office only" (type Error).</t>
         </is>
       </c>
       <c r="F37" s="24" t="inlineStr">
@@ -14959,12 +14959,12 @@
     <row r="38">
       <c r="A38" s="22" t="inlineStr">
         <is>
-          <t>M-036</t>
+          <t>M-066</t>
         </is>
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
+          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
         </is>
       </c>
       <c r="C38" s="22" t="inlineStr">
@@ -14979,7 +14979,7 @@
       </c>
       <c r="E38" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the gross amount" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "An official receipt needs a line" (type Error).</t>
         </is>
       </c>
       <c r="F38" s="22" t="inlineStr">
@@ -15012,12 +15012,12 @@
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>M-037</t>
+          <t>M-067</t>
         </is>
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
+          <t>Receive Payment (SCR-OP-08) and the application of payments</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
@@ -15032,7 +15032,7 @@
       </c>
       <c r="E39" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Payor name is required" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A receipt needs an amount above zero" (type Error).</t>
         </is>
       </c>
       <c r="F39" s="24" t="inlineStr">
@@ -15065,7 +15065,7 @@
     <row r="40">
       <c r="A40" s="22" t="inlineStr">
         <is>
-          <t>M-038</t>
+          <t>M-068</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
@@ -15085,7 +15085,7 @@
       </c>
       <c r="E40" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Select the OR type" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;receipt no&gt; issued" (type Confirmation).</t>
         </is>
       </c>
       <c r="F40" s="22" t="inlineStr">
@@ -15118,7 +15118,7 @@
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>M-039</t>
+          <t>M-069</t>
         </is>
       </c>
       <c r="B41" s="24" t="inlineStr">
@@ -15138,7 +15138,7 @@
       </c>
       <c r="E41" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "VAT and withholding tax cannot be negative" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the gross amount" (type Validation).</t>
         </is>
       </c>
       <c r="F41" s="24" t="inlineStr">
@@ -15171,7 +15171,7 @@
     <row r="42">
       <c r="A42" s="22" t="inlineStr">
         <is>
-          <t>M-040</t>
+          <t>M-070</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
@@ -15191,7 +15191,7 @@
       </c>
       <c r="E42" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Branch &lt;code&gt; is not of this company" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No receipts match the search" (type Information).</t>
         </is>
       </c>
       <c r="F42" s="22" t="inlineStr">
@@ -15224,7 +15224,7 @@
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>M-041</t>
+          <t>M-071</t>
         </is>
       </c>
       <c r="B43" s="24" t="inlineStr">
@@ -15244,7 +15244,7 @@
       </c>
       <c r="E43" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The company has no Head Office branch for official receipts" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Payor name is required" (type Validation).</t>
         </is>
       </c>
       <c r="F43" s="24" t="inlineStr">
@@ -15277,7 +15277,7 @@
     <row r="44">
       <c r="A44" s="22" t="inlineStr">
         <is>
-          <t>M-042</t>
+          <t>M-072</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="E44" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Official receipt series belong to Head Office only" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Select the OR type" (type Validation).</t>
         </is>
       </c>
       <c r="F44" s="22" t="inlineStr">
@@ -15330,7 +15330,7 @@
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>M-043</t>
+          <t>M-073</t>
         </is>
       </c>
       <c r="B45" s="24" t="inlineStr">
@@ -15350,7 +15350,7 @@
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No authorized &lt;kind&gt; series with numbers left for this branch" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "VAT and withholding tax cannot be negative" (type Validation).</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
@@ -15383,7 +15383,7 @@
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
-          <t>M-044</t>
+          <t>M-074</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -15403,7 +15403,7 @@
       </c>
       <c r="E46" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt series &lt;prefix&gt; is depleted" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Branch &lt;code&gt; is not of this company" (type Error).</t>
         </is>
       </c>
       <c r="F46" s="22" t="inlineStr">
@@ -15436,7 +15436,7 @@
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>M-045</t>
+          <t>M-075</t>
         </is>
       </c>
       <c r="B47" s="24" t="inlineStr">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="E47" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Next number &lt;legacy next no&gt; is outside &lt;from no&gt;-&lt;to no&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The company has no Head Office branch for official receipts" (type Error).</t>
         </is>
       </c>
       <c r="F47" s="24" t="inlineStr">
@@ -15489,7 +15489,7 @@
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>M-046</t>
+          <t>M-076</t>
         </is>
       </c>
       <c r="B48" s="22" t="inlineStr">
@@ -15509,7 +15509,7 @@
       </c>
       <c r="E48" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The last number cannot be below the numbers already issued" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Official receipt series belong to Head Office only" (type Error).</t>
         </is>
       </c>
       <c r="F48" s="22" t="inlineStr">
@@ -15542,7 +15542,7 @@
     <row r="49">
       <c r="A49" s="24" t="inlineStr">
         <is>
-          <t>M-047</t>
+          <t>M-077</t>
         </is>
       </c>
       <c r="B49" s="24" t="inlineStr">
@@ -15562,7 +15562,7 @@
       </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The last number must not be below the first number" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No authorized &lt;kind&gt; series with numbers left for this branch" (type Error).</t>
         </is>
       </c>
       <c r="F49" s="24" t="inlineStr">
@@ -15595,12 +15595,12 @@
     <row r="50">
       <c r="A50" s="22" t="inlineStr">
         <is>
-          <t>M-048</t>
+          <t>M-078</t>
         </is>
       </c>
       <c r="B50" s="22" t="inlineStr">
         <is>
-          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
+          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
         </is>
       </c>
       <c r="C50" s="22" t="inlineStr">
@@ -15615,7 +15615,7 @@
       </c>
       <c r="E50" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No cancellation or reinstatement" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt series &lt;prefix&gt; is depleted" (type Error).</t>
         </is>
       </c>
       <c r="F50" s="22" t="inlineStr">
@@ -15648,12 +15648,12 @@
     <row r="51">
       <c r="A51" s="24" t="inlineStr">
         <is>
-          <t>M-049</t>
+          <t>M-079</t>
         </is>
       </c>
       <c r="B51" s="24" t="inlineStr">
         <is>
-          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
+          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
         </is>
       </c>
       <c r="C51" s="24" t="inlineStr">
@@ -15668,7 +15668,7 @@
       </c>
       <c r="E51" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No items to display" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Next number &lt;legacy next no&gt; is outside &lt;from no&gt;-&lt;to no&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F51" s="24" t="inlineStr">
@@ -15701,12 +15701,12 @@
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>M-050</t>
+          <t>M-080</t>
         </is>
       </c>
       <c r="B52" s="22" t="inlineStr">
         <is>
-          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
+          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
         </is>
       </c>
       <c r="C52" s="22" t="inlineStr">
@@ -15721,7 +15721,7 @@
       </c>
       <c r="E52" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No journal posted yet" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The last number cannot be below the numbers already issued" (type Error).</t>
         </is>
       </c>
       <c r="F52" s="22" t="inlineStr">
@@ -15754,12 +15754,12 @@
     <row r="53">
       <c r="A53" s="24" t="inlineStr">
         <is>
-          <t>M-051</t>
+          <t>M-081</t>
         </is>
       </c>
       <c r="B53" s="24" t="inlineStr">
         <is>
-          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
+          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
         </is>
       </c>
       <c r="C53" s="24" t="inlineStr">
@@ -15774,7 +15774,7 @@
       </c>
       <c r="E53" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Nothing applied from this receipt" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The last number must not be below the first number" (type Error).</t>
         </is>
       </c>
       <c r="F53" s="24" t="inlineStr">
@@ -15807,12 +15807,12 @@
     <row r="54">
       <c r="A54" s="22" t="inlineStr">
         <is>
-          <t>M-052</t>
+          <t>M-082</t>
         </is>
       </c>
       <c r="B54" s="22" t="inlineStr">
         <is>
-          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
+          <t>Receipts, Issue Official Receipt and the receipt series (SCR</t>
         </is>
       </c>
       <c r="C54" s="22" t="inlineStr">
@@ -15827,7 +15827,7 @@
       </c>
       <c r="E54" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The requested action is applied to the receipt." (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The number format must hold the sequence {SEQ}" (type Error).</t>
         </is>
       </c>
       <c r="F54" s="22" t="inlineStr">
@@ -15860,7 +15860,7 @@
     <row r="55">
       <c r="A55" s="24" t="inlineStr">
         <is>
-          <t>M-053</t>
+          <t>M-083</t>
         </is>
       </c>
       <c r="B55" s="24" t="inlineStr">
@@ -15880,7 +15880,7 @@
       </c>
       <c r="E55" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve &lt;transaction no&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No cancellation or reinstatement" (type Information).</t>
         </is>
       </c>
       <c r="F55" s="24" t="inlineStr">
@@ -15913,7 +15913,7 @@
     <row r="56">
       <c r="A56" s="22" t="inlineStr">
         <is>
-          <t>M-054</t>
+          <t>M-084</t>
         </is>
       </c>
       <c r="B56" s="22" t="inlineStr">
@@ -15933,7 +15933,7 @@
       </c>
       <c r="E56" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;transaction no&gt; is &lt;stage&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No items to display" (type Information).</t>
         </is>
       </c>
       <c r="F56" s="22" t="inlineStr">
@@ -15966,7 +15966,7 @@
     <row r="57">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>M-055</t>
+          <t>M-085</t>
         </is>
       </c>
       <c r="B57" s="24" t="inlineStr">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="E57" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; already has a request waiting for approval" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No journal posted yet" (type Information).</t>
         </is>
       </c>
       <c r="F57" s="24" t="inlineStr">
@@ -16019,7 +16019,7 @@
     <row r="58">
       <c r="A58" s="22" t="inlineStr">
         <is>
-          <t>M-056</t>
+          <t>M-086</t>
         </is>
       </c>
       <c r="B58" s="22" t="inlineStr">
@@ -16039,7 +16039,7 @@
       </c>
       <c r="E58" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; is already cancelled" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Nothing applied from this receipt" (type Information).</t>
         </is>
       </c>
       <c r="F58" s="22" t="inlineStr">
@@ -16072,7 +16072,7 @@
     <row r="59">
       <c r="A59" s="24" t="inlineStr">
         <is>
-          <t>M-057</t>
+          <t>M-087</t>
         </is>
       </c>
       <c r="B59" s="24" t="inlineStr">
@@ -16092,7 +16092,7 @@
       </c>
       <c r="E59" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unapplied item &lt;reference&gt; of the receipt is &lt;stage&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The requested action is applied to the receipt." (type Validation).</t>
         </is>
       </c>
       <c r="F59" s="24" t="inlineStr">
@@ -16125,7 +16125,7 @@
     <row r="60">
       <c r="A60" s="22" t="inlineStr">
         <is>
-          <t>M-058</t>
+          <t>M-088</t>
         </is>
       </c>
       <c r="B60" s="22" t="inlineStr">
@@ -16145,7 +16145,7 @@
       </c>
       <c r="E60" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Only a cancelled receipt can be reinstated" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve &lt;transaction no&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F60" s="22" t="inlineStr">
@@ -16178,7 +16178,7 @@
     <row r="61">
       <c r="A61" s="24" t="inlineStr">
         <is>
-          <t>M-059</t>
+          <t>M-089</t>
         </is>
       </c>
       <c r="B61" s="24" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="E61" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Select a reason" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;transaction no&gt; is &lt;stage&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F61" s="24" t="inlineStr">
@@ -16231,7 +16231,7 @@
     <row r="62">
       <c r="A62" s="22" t="inlineStr">
         <is>
-          <t>M-060</t>
+          <t>M-090</t>
         </is>
       </c>
       <c r="B62" s="22" t="inlineStr">
@@ -16251,7 +16251,7 @@
       </c>
       <c r="E62" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Specify the reason when 'Others' is selected" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; already has a request waiting for approval" (type Error).</t>
         </is>
       </c>
       <c r="F62" s="22" t="inlineStr">
@@ -16284,7 +16284,7 @@
     <row r="63">
       <c r="A63" s="24" t="inlineStr">
         <is>
-          <t>M-061</t>
+          <t>M-091</t>
         </is>
       </c>
       <c r="B63" s="24" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="E63" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The reinstated amount must be above zero and at most &lt;amount&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; is already cancelled" (type Error).</t>
         </is>
       </c>
       <c r="F63" s="24" t="inlineStr">
@@ -16337,7 +16337,7 @@
     <row r="64">
       <c r="A64" s="22" t="inlineStr">
         <is>
-          <t>M-062</t>
+          <t>M-092</t>
         </is>
       </c>
       <c r="B64" s="22" t="inlineStr">
@@ -16357,7 +16357,7 @@
       </c>
       <c r="E64" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the &lt;missing&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unapplied item &lt;reference&gt; of the receipt is &lt;stage&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F64" s="22" t="inlineStr">
@@ -16390,7 +16390,7 @@
     <row r="65">
       <c r="A65" s="24" t="inlineStr">
         <is>
-          <t>M-063</t>
+          <t>M-093</t>
         </is>
       </c>
       <c r="B65" s="24" t="inlineStr">
@@ -16410,7 +16410,7 @@
       </c>
       <c r="E65" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Premium reinstatement reasons apply to ARs" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Only a cancelled receipt can be reinstated" (type Error).</t>
         </is>
       </c>
       <c r="F65" s="24" t="inlineStr">
@@ -16443,12 +16443,12 @@
     <row r="66">
       <c r="A66" s="22" t="inlineStr">
         <is>
-          <t>M-064</t>
+          <t>M-094</t>
         </is>
       </c>
       <c r="B66" s="22" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C66" s="22" t="inlineStr">
@@ -16463,7 +16463,7 @@
       </c>
       <c r="E66" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition updated" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Select a reason" (type Error).</t>
         </is>
       </c>
       <c r="F66" s="22" t="inlineStr">
@@ -16496,12 +16496,12 @@
     <row r="67">
       <c r="A67" s="24" t="inlineStr">
         <is>
-          <t>M-065</t>
+          <t>M-095</t>
         </is>
       </c>
       <c r="B67" s="24" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C67" s="24" t="inlineStr">
@@ -16516,7 +16516,7 @@
       </c>
       <c r="E67" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No disposition yet" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Specify the reason when 'Others' is selected" (type Error).</t>
         </is>
       </c>
       <c r="F67" s="24" t="inlineStr">
@@ -16549,12 +16549,12 @@
     <row r="68">
       <c r="A68" s="22" t="inlineStr">
         <is>
-          <t>M-066</t>
+          <t>M-096</t>
         </is>
       </c>
       <c r="B68" s="22" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C68" s="22" t="inlineStr">
@@ -16569,7 +16569,7 @@
       </c>
       <c r="E68" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The amount must be above zero and at most the balance &lt;balance&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The reinstated amount must be above zero and at most &lt;amount&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F68" s="22" t="inlineStr">
@@ -16602,12 +16602,12 @@
     <row r="69">
       <c r="A69" s="24" t="inlineStr">
         <is>
-          <t>M-067</t>
+          <t>M-097</t>
         </is>
       </c>
       <c r="B69" s="24" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C69" s="24" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="E69" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Invoice &lt;invoice no&gt; takes no client payment" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the &lt;missing&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F69" s="24" t="inlineStr">
@@ -16655,12 +16655,12 @@
     <row r="70">
       <c r="A70" s="22" t="inlineStr">
         <is>
-          <t>M-068</t>
+          <t>M-098</t>
         </is>
       </c>
       <c r="B70" s="22" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C70" s="22" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="E70" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown invoice &lt;invoice no&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Premium reinstatement reasons apply to ARs" (type Error).</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
@@ -16708,12 +16708,12 @@
     <row r="71">
       <c r="A71" s="24" t="inlineStr">
         <is>
-          <t>M-069</t>
+          <t>M-099</t>
         </is>
       </c>
       <c r="B71" s="24" t="inlineStr">
         <is>
-          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
+          <t>Receipt: cancellation and reinstatement (SCR-OP-10)</t>
         </is>
       </c>
       <c r="C71" s="24" t="inlineStr">
@@ -16728,7 +16728,7 @@
       </c>
       <c r="E71" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;description&gt; needs the team leader's approval and is not processed at once" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Reinstatement of a cancelled receipt is not enabled (setting What Reinstate does)" (type Error).</t>
         </is>
       </c>
       <c r="F71" s="24" t="inlineStr">
@@ -16761,7 +16761,7 @@
     <row r="72">
       <c r="A72" s="22" t="inlineStr">
         <is>
-          <t>M-070</t>
+          <t>M-100</t>
         </is>
       </c>
       <c r="B72" s="22" t="inlineStr">
@@ -16781,7 +16781,7 @@
       </c>
       <c r="E72" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Invoice &lt;target invoice no&gt; has nothing outstanding to apply to" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition updated" (type Confirmation).</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
@@ -16814,7 +16814,7 @@
     <row r="73">
       <c r="A73" s="24" t="inlineStr">
         <is>
-          <t>M-071</t>
+          <t>M-101</t>
         </is>
       </c>
       <c r="B73" s="24" t="inlineStr">
@@ -16834,7 +16834,7 @@
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No application" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No disposition yet" (type Information).</t>
         </is>
       </c>
       <c r="F73" s="24" t="inlineStr">
@@ -16867,7 +16867,7 @@
     <row r="74">
       <c r="A74" s="22" t="inlineStr">
         <is>
-          <t>M-072</t>
+          <t>M-102</t>
         </is>
       </c>
       <c r="B74" s="22" t="inlineStr">
@@ -16887,7 +16887,7 @@
       </c>
       <c r="E74" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter &lt;what&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No unapplied payment matches the filters." (type Information).</t>
         </is>
       </c>
       <c r="F74" s="22" t="inlineStr">
@@ -16920,7 +16920,7 @@
     <row r="75">
       <c r="A75" s="24" t="inlineStr">
         <is>
-          <t>M-073</t>
+          <t>M-103</t>
         </is>
       </c>
       <c r="B75" s="24" t="inlineStr">
@@ -16940,7 +16940,7 @@
       </c>
       <c r="E75" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition type &lt;type code&gt; has no processing rule" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The amount must be above zero and at most the balance &lt;balance&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F75" s="24" t="inlineStr">
@@ -16973,7 +16973,7 @@
     <row r="76">
       <c r="A76" s="22" t="inlineStr">
         <is>
-          <t>M-074</t>
+          <t>M-104</t>
         </is>
       </c>
       <c r="B76" s="22" t="inlineStr">
@@ -16993,7 +16993,7 @@
       </c>
       <c r="E76" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A reclass or transfer moves the whole balance &lt;balance&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Invoice &lt;invoice no&gt; takes no client payment" (type Error).</t>
         </is>
       </c>
       <c r="F76" s="22" t="inlineStr">
@@ -17026,7 +17026,7 @@
     <row r="77">
       <c r="A77" s="24" t="inlineStr">
         <is>
-          <t>M-075</t>
+          <t>M-105</t>
         </is>
       </c>
       <c r="B77" s="24" t="inlineStr">
@@ -17046,7 +17046,7 @@
       </c>
       <c r="E77" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve the disposition" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown invoice &lt;invoice no&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F77" s="24" t="inlineStr">
@@ -17079,7 +17079,7 @@
     <row r="78">
       <c r="A78" s="22" t="inlineStr">
         <is>
-          <t>M-076</t>
+          <t>M-106</t>
         </is>
       </c>
       <c r="B78" s="22" t="inlineStr">
@@ -17099,7 +17099,7 @@
       </c>
       <c r="E78" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A refund is reversed only after Disbursement returned the request" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;description&gt; needs the team leader's approval and is not processed at once" (type Error).</t>
         </is>
       </c>
       <c r="F78" s="22" t="inlineStr">
@@ -17132,7 +17132,7 @@
     <row r="79">
       <c r="A79" s="24" t="inlineStr">
         <is>
-          <t>M-077</t>
+          <t>M-107</t>
         </is>
       </c>
       <c r="B79" s="24" t="inlineStr">
@@ -17152,7 +17152,7 @@
       </c>
       <c r="E79" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the reason for the reversal" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Invoice &lt;target invoice no&gt; has nothing outstanding to apply to" (type Error).</t>
         </is>
       </c>
       <c r="F79" s="24" t="inlineStr">
@@ -17185,7 +17185,7 @@
     <row r="80">
       <c r="A80" s="22" t="inlineStr">
         <is>
-          <t>M-078</t>
+          <t>M-108</t>
         </is>
       </c>
       <c r="B80" s="22" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="E80" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "An unapplied item needs an amount above zero" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No application" (type Error).</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
@@ -17238,7 +17238,7 @@
     <row r="81">
       <c r="A81" s="24" t="inlineStr">
         <is>
-          <t>M-079</t>
+          <t>M-109</t>
         </is>
       </c>
       <c r="B81" s="24" t="inlineStr">
@@ -17258,7 +17258,7 @@
       </c>
       <c r="E81" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Amount &lt;value&gt; is above the unapplied balance &lt;balance&gt; of &lt;reference&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter &lt;what&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F81" s="24" t="inlineStr">
@@ -17291,7 +17291,7 @@
     <row r="82">
       <c r="A82" s="22" t="inlineStr">
         <is>
-          <t>M-080</t>
+          <t>M-110</t>
         </is>
       </c>
       <c r="B82" s="22" t="inlineStr">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="E82" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;reference&gt; is &lt;stage&gt;, not &lt;stage&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition type &lt;type code&gt; has no processing rule" (type Error).</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
@@ -17344,12 +17344,12 @@
     <row r="83">
       <c r="A83" s="24" t="inlineStr">
         <is>
-          <t>M-081</t>
+          <t>M-111</t>
         </is>
       </c>
       <c r="B83" s="24" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C83" s="24" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="E83" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most the unapplied balance" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A reclass or transfer moves the whole balance &lt;balance&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F83" s="24" t="inlineStr">
@@ -17397,12 +17397,12 @@
     <row r="84">
       <c r="A84" s="22" t="inlineStr">
         <is>
-          <t>M-082</t>
+          <t>M-112</t>
         </is>
       </c>
       <c r="B84" s="22" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C84" s="22" t="inlineStr">
@@ -17417,7 +17417,7 @@
       </c>
       <c r="E84" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the client to reclass to" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve the disposition" (type Error).</t>
         </is>
       </c>
       <c r="F84" s="22" t="inlineStr">
@@ -17450,12 +17450,12 @@
     <row r="85">
       <c r="A85" s="24" t="inlineStr">
         <is>
-          <t>M-083</t>
+          <t>M-113</t>
         </is>
       </c>
       <c r="B85" s="24" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C85" s="24" t="inlineStr">
@@ -17470,7 +17470,7 @@
       </c>
       <c r="E85" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the marketing unit to transfer to" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A refund is reversed only after Disbursement returned the request" (type Error).</t>
         </is>
       </c>
       <c r="F85" s="24" t="inlineStr">
@@ -17503,12 +17503,12 @@
     <row r="86">
       <c r="A86" s="22" t="inlineStr">
         <is>
-          <t>M-084</t>
+          <t>M-114</t>
         </is>
       </c>
       <c r="B86" s="22" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C86" s="22" t="inlineStr">
@@ -17523,7 +17523,7 @@
       </c>
       <c r="E86" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No collector requests to display" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the reason for the reversal" (type Error).</t>
         </is>
       </c>
       <c r="F86" s="22" t="inlineStr">
@@ -17556,12 +17556,12 @@
     <row r="87">
       <c r="A87" s="24" t="inlineStr">
         <is>
-          <t>M-085</t>
+          <t>M-115</t>
         </is>
       </c>
       <c r="B87" s="24" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
@@ -17576,7 +17576,7 @@
       </c>
       <c r="E87" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No payment reversals to display" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "An unapplied item needs an amount above zero" (type Error).</t>
         </is>
       </c>
       <c r="F87" s="24" t="inlineStr">
@@ -17609,12 +17609,12 @@
     <row r="88">
       <c r="A88" s="22" t="inlineStr">
         <is>
-          <t>M-086</t>
+          <t>M-116</t>
         </is>
       </c>
       <c r="B88" s="22" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C88" s="22" t="inlineStr">
@@ -17629,7 +17629,7 @@
       </c>
       <c r="E88" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No refund validations to display" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Amount &lt;value&gt; is above the unapplied balance &lt;balance&gt; of &lt;reference&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F88" s="22" t="inlineStr">
@@ -17662,12 +17662,12 @@
     <row r="89">
       <c r="A89" s="24" t="inlineStr">
         <is>
-          <t>M-087</t>
+          <t>M-117</t>
         </is>
       </c>
       <c r="B89" s="24" t="inlineStr">
         <is>
-          <t>Incoming Requests (SCR-OP-13)</t>
+          <t>Unapplied Payments and dispositions (SCR-OP-11, SCR-OP-12)</t>
         </is>
       </c>
       <c r="C89" s="24" t="inlineStr">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="E89" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The selected receipt is reversed as requested." (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;reference&gt; is &lt;stage&gt;, not &lt;stage&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F89" s="24" t="inlineStr">
@@ -17715,7 +17715,7 @@
     <row r="90">
       <c r="A90" s="22" t="inlineStr">
         <is>
-          <t>M-088</t>
+          <t>M-118</t>
         </is>
       </c>
       <c r="B90" s="22" t="inlineStr">
@@ -17735,7 +17735,7 @@
       </c>
       <c r="E90" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;request no&gt; is already &lt;status&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero and at most the unapplied balance" (type Validation).</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -17768,7 +17768,7 @@
     <row r="91">
       <c r="A91" s="24" t="inlineStr">
         <is>
-          <t>M-089</t>
+          <t>M-119</t>
         </is>
       </c>
       <c r="B91" s="24" t="inlineStr">
@@ -17788,7 +17788,7 @@
       </c>
       <c r="E91" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition type &lt;type&gt; does not carry out a &lt;action&gt; request" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the client to reclass to" (type Validation).</t>
         </is>
       </c>
       <c r="F91" s="24" t="inlineStr">
@@ -17821,7 +17821,7 @@
     <row r="92">
       <c r="A92" s="22" t="inlineStr">
         <is>
-          <t>M-090</t>
+          <t>M-120</t>
         </is>
       </c>
       <c r="B92" s="22" t="inlineStr">
@@ -17841,7 +17841,7 @@
       </c>
       <c r="E92" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown disposition type &lt;type&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the marketing unit to transfer to" (type Validation).</t>
         </is>
       </c>
       <c r="F92" s="22" t="inlineStr">
@@ -17874,7 +17874,7 @@
     <row r="93">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>M-091</t>
+          <t>M-121</t>
         </is>
       </c>
       <c r="B93" s="24" t="inlineStr">
@@ -17894,7 +17894,7 @@
       </c>
       <c r="E93" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve the payment reversal" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No collector requests to display" (type Information).</t>
         </is>
       </c>
       <c r="F93" s="24" t="inlineStr">
@@ -17927,7 +17927,7 @@
     <row r="94">
       <c r="A94" s="22" t="inlineStr">
         <is>
-          <t>M-092</t>
+          <t>M-122</t>
         </is>
       </c>
       <c r="B94" s="22" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="E94" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;request no&gt; is already &lt;status&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No payment reversals to display" (type Information).</t>
         </is>
       </c>
       <c r="F94" s="22" t="inlineStr">
@@ -17980,7 +17980,7 @@
     <row r="95">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>M-093</t>
+          <t>M-123</t>
         </is>
       </c>
       <c r="B95" s="24" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="E95" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; has &lt;available&gt; applied to &lt;invoice no&gt;, less than &lt;target&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No refund validations to display" (type Information).</t>
         </is>
       </c>
       <c r="F95" s="24" t="inlineStr">
@@ -18033,7 +18033,7 @@
     <row r="96">
       <c r="A96" s="22" t="inlineStr">
         <is>
-          <t>M-094</t>
+          <t>M-124</t>
         </is>
       </c>
       <c r="B96" s="22" t="inlineStr">
@@ -18053,7 +18053,7 @@
       </c>
       <c r="E96" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown receipt &lt;receipt no&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The selected receipt is reversed as requested." (type Validation).</t>
         </is>
       </c>
       <c r="F96" s="22" t="inlineStr">
@@ -18086,7 +18086,7 @@
     <row r="97">
       <c r="A97" s="24" t="inlineStr">
         <is>
-          <t>M-095</t>
+          <t>M-125</t>
         </is>
       </c>
       <c r="B97" s="24" t="inlineStr">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="E97" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;task no&gt; is already &lt;status&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;request no&gt; is already &lt;status&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F97" s="24" t="inlineStr">
@@ -18139,7 +18139,7 @@
     <row r="98">
       <c r="A98" s="22" t="inlineStr">
         <is>
-          <t>M-096</t>
+          <t>M-126</t>
         </is>
       </c>
       <c r="B98" s="22" t="inlineStr">
@@ -18159,7 +18159,7 @@
       </c>
       <c r="E98" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Choose the unapplied item that holds the returned premium" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Disposition type &lt;type&gt; does not carry out a &lt;action&gt; request" (type Error).</t>
         </is>
       </c>
       <c r="F98" s="22" t="inlineStr">
@@ -18192,7 +18192,7 @@
     <row r="99">
       <c r="A99" s="24" t="inlineStr">
         <is>
-          <t>M-097</t>
+          <t>M-127</t>
         </is>
       </c>
       <c r="B99" s="24" t="inlineStr">
@@ -18212,7 +18212,7 @@
       </c>
       <c r="E99" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the reason for rejecting" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown disposition type &lt;type&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F99" s="24" t="inlineStr">
@@ -18245,12 +18245,12 @@
     <row r="100">
       <c r="A100" s="22" t="inlineStr">
         <is>
-          <t>M-098</t>
+          <t>M-128</t>
         </is>
       </c>
       <c r="B100" s="22" t="inlineStr">
         <is>
-          <t>Pre-booked Payments (SCR-OP-14)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C100" s="22" t="inlineStr">
@@ -18265,7 +18265,7 @@
       </c>
       <c r="E100" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No items to display" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The requester cannot approve the payment reversal" (type Error).</t>
         </is>
       </c>
       <c r="F100" s="22" t="inlineStr">
@@ -18298,12 +18298,12 @@
     <row r="101">
       <c r="A101" s="24" t="inlineStr">
         <is>
-          <t>M-099</t>
+          <t>M-129</t>
         </is>
       </c>
       <c r="B101" s="24" t="inlineStr">
         <is>
-          <t>Pre-booked Payments (SCR-OP-14)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
@@ -18318,7 +18318,7 @@
       </c>
       <c r="E101" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Pre-booked payment of &lt;arn&gt; is &lt;status&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;request no&gt; is already &lt;status&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F101" s="24" t="inlineStr">
@@ -18351,12 +18351,12 @@
     <row r="102">
       <c r="A102" s="22" t="inlineStr">
         <is>
-          <t>M-100</t>
+          <t>M-130</t>
         </is>
       </c>
       <c r="B102" s="22" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C102" s="22" t="inlineStr">
@@ -18371,7 +18371,7 @@
       </c>
       <c r="E102" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Layout of &lt;handler code&gt; saved" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; has &lt;available&gt; applied to &lt;invoice no&gt;, less than &lt;target&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F102" s="22" t="inlineStr">
@@ -18404,12 +18404,12 @@
     <row r="103">
       <c r="A103" s="24" t="inlineStr">
         <is>
-          <t>M-101</t>
+          <t>M-131</t>
         </is>
       </c>
       <c r="B103" s="24" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C103" s="24" t="inlineStr">
@@ -18424,7 +18424,7 @@
       </c>
       <c r="E103" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No payment accepted in this run" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown receipt &lt;receipt no&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F103" s="24" t="inlineStr">
@@ -18457,12 +18457,12 @@
     <row r="104">
       <c r="A104" s="22" t="inlineStr">
         <is>
-          <t>M-102</t>
+          <t>M-132</t>
         </is>
       </c>
       <c r="B104" s="22" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C104" s="22" t="inlineStr">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="E104" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Sweep done: &lt;premium&gt; premium balance(s) reversed, &lt;excess&gt; excess moved to overages" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;task no&gt; is already &lt;status&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F104" s="22" t="inlineStr">
@@ -18510,12 +18510,12 @@
     <row r="105">
       <c r="A105" s="24" t="inlineStr">
         <is>
-          <t>M-103</t>
+          <t>M-133</t>
         </is>
       </c>
       <c r="B105" s="24" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C105" s="24" t="inlineStr">
@@ -18530,7 +18530,7 @@
       </c>
       <c r="E105" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A delimited layout needs a one-character separator" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Choose the unapplied item that holds the returned premium" (type Error).</t>
         </is>
       </c>
       <c r="F105" s="24" t="inlineStr">
@@ -18563,12 +18563,12 @@
     <row r="106">
       <c r="A106" s="22" t="inlineStr">
         <is>
-          <t>M-104</t>
+          <t>M-134</t>
         </is>
       </c>
       <c r="B106" s="22" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Incoming Requests (SCR-OP-13)</t>
         </is>
       </c>
       <c r="C106" s="22" t="inlineStr">
@@ -18583,7 +18583,7 @@
       </c>
       <c r="E106" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A fixed-width layout needs its fields" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the reason for rejecting" (type Error).</t>
         </is>
       </c>
       <c r="F106" s="22" t="inlineStr">
@@ -18616,12 +18616,12 @@
     <row r="107">
       <c r="A107" s="24" t="inlineStr">
         <is>
-          <t>M-105</t>
+          <t>M-135</t>
         </is>
       </c>
       <c r="B107" s="24" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Pre-booked Payments (SCR-OP-14)</t>
         </is>
       </c>
       <c r="C107" s="24" t="inlineStr">
@@ -18636,7 +18636,7 @@
       </c>
       <c r="E107" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Start and length of '&lt;part&gt;' must be numbers" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No items to display" (type Information).</t>
         </is>
       </c>
       <c r="F107" s="24" t="inlineStr">
@@ -18669,12 +18669,12 @@
     <row r="108">
       <c r="A108" s="22" t="inlineStr">
         <is>
-          <t>M-106</t>
+          <t>M-136</t>
         </is>
       </c>
       <c r="B108" s="22" t="inlineStr">
         <is>
-          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
+          <t>Pre-booked Payments (SCR-OP-14)</t>
         </is>
       </c>
       <c r="C108" s="22" t="inlineStr">
@@ -18689,7 +18689,7 @@
       </c>
       <c r="E108" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Write each field as Header:start:length, not '&lt;part&gt;'" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Pre-booked payment of &lt;arn&gt; is &lt;status&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F108" s="22" t="inlineStr">
@@ -18722,7 +18722,7 @@
     <row r="109">
       <c r="A109" s="24" t="inlineStr">
         <is>
-          <t>M-107</t>
+          <t>M-137</t>
         </is>
       </c>
       <c r="B109" s="24" t="inlineStr">
@@ -18742,7 +18742,7 @@
       </c>
       <c r="E109" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown layout kind &lt;new kind&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Layout of &lt;handler code&gt; saved" (type Confirmation).</t>
         </is>
       </c>
       <c r="F109" s="24" t="inlineStr">
@@ -18775,12 +18775,12 @@
     <row r="110">
       <c r="A110" s="22" t="inlineStr">
         <is>
-          <t>M-108</t>
+          <t>M-138</t>
         </is>
       </c>
       <c r="B110" s="22" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C110" s="22" t="inlineStr">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="E110" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No payment accepted in this run" (type Information).</t>
         </is>
       </c>
       <c r="F110" s="22" t="inlineStr">
@@ -18828,12 +18828,12 @@
     <row r="111">
       <c r="A111" s="24" t="inlineStr">
         <is>
-          <t>M-109</t>
+          <t>M-139</t>
         </is>
       </c>
       <c r="B111" s="24" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C111" s="24" t="inlineStr">
@@ -18848,7 +18848,7 @@
       </c>
       <c r="E111" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "PDC warehouse updated" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Sweep done: &lt;premium&gt; reversed, &lt;excess&gt; excess moved to overages" (type Confirmation).</t>
         </is>
       </c>
       <c r="F111" s="24" t="inlineStr">
@@ -18881,12 +18881,12 @@
     <row r="112">
       <c r="A112" s="22" t="inlineStr">
         <is>
-          <t>M-110</t>
+          <t>M-140</t>
         </is>
       </c>
       <c r="B112" s="22" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C112" s="22" t="inlineStr">
@@ -18901,7 +18901,7 @@
       </c>
       <c r="E112" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A post-dated check needs an amount above zero" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A delimited layout needs a one-character separator" (type Error).</t>
         </is>
       </c>
       <c r="F112" s="22" t="inlineStr">
@@ -18934,12 +18934,12 @@
     <row r="113">
       <c r="A113" s="24" t="inlineStr">
         <is>
-          <t>M-111</t>
+          <t>M-141</t>
         </is>
       </c>
       <c r="B113" s="24" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C113" s="24" t="inlineStr">
@@ -18954,7 +18954,7 @@
       </c>
       <c r="E113" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Check &lt;bank code&gt; &lt;check no&gt; is already warehoused" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A fixed-width layout needs its fields" (type Error).</t>
         </is>
       </c>
       <c r="F113" s="24" t="inlineStr">
@@ -18987,12 +18987,12 @@
     <row r="114">
       <c r="A114" s="22" t="inlineStr">
         <is>
-          <t>M-112</t>
+          <t>M-142</t>
         </is>
       </c>
       <c r="B114" s="22" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C114" s="22" t="inlineStr">
@@ -19007,7 +19007,7 @@
       </c>
       <c r="E114" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Check &lt;warehouse no&gt; is &lt;status&gt;, not in the warehouse" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Start and length of '&lt;part&gt;' must be numbers" (type Error).</t>
         </is>
       </c>
       <c r="F114" s="22" t="inlineStr">
@@ -19040,12 +19040,12 @@
     <row r="115">
       <c r="A115" s="24" t="inlineStr">
         <is>
-          <t>M-113</t>
+          <t>M-143</t>
         </is>
       </c>
       <c r="B115" s="24" t="inlineStr">
         <is>
-          <t>PDC Warehouse (SCR-OP-16)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C115" s="24" t="inlineStr">
@@ -19060,7 +19060,7 @@
       </c>
       <c r="E115" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "A check leaves the warehouse as returned, replaced or pulled out" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Write each field as Header:start:length, not '&lt;part&gt;'" (type Error).</t>
         </is>
       </c>
       <c r="F115" s="24" t="inlineStr">
@@ -19093,12 +19093,12 @@
     <row r="116">
       <c r="A116" s="22" t="inlineStr">
         <is>
-          <t>M-114</t>
+          <t>M-144</t>
         </is>
       </c>
       <c r="B116" s="22" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>Payment Uploads and Cashiering Setup (SCR-OP-15, SCR-OP-22)</t>
         </is>
       </c>
       <c r="C116" s="22" t="inlineStr">
@@ -19113,7 +19113,7 @@
       </c>
       <c r="E116" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt;: &lt;printed count&gt; printed, &lt;failed count&gt; failed" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown layout kind &lt;new kind&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F116" s="22" t="inlineStr">
@@ -19146,12 +19146,12 @@
     <row r="117">
       <c r="A117" s="24" t="inlineStr">
         <is>
-          <t>M-115</t>
+          <t>M-145</t>
         </is>
       </c>
       <c r="B117" s="24" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C117" s="24" t="inlineStr">
@@ -19166,7 +19166,7 @@
       </c>
       <c r="E117" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No print batch yet" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter an amount above zero" (type Validation).</t>
         </is>
       </c>
       <c r="F117" s="24" t="inlineStr">
@@ -19199,12 +19199,12 @@
     <row r="118">
       <c r="A118" s="22" t="inlineStr">
         <is>
-          <t>M-116</t>
+          <t>M-146</t>
         </is>
       </c>
       <c r="B118" s="22" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C118" s="22" t="inlineStr">
@@ -19219,7 +19219,7 @@
       </c>
       <c r="E118" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No receipts match the criteria" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No post-dated checks" (type Information).</t>
         </is>
       </c>
       <c r="F118" s="22" t="inlineStr">
@@ -19252,12 +19252,12 @@
     <row r="119">
       <c r="A119" s="24" t="inlineStr">
         <is>
-          <t>M-117</t>
+          <t>M-147</t>
         </is>
       </c>
       <c r="B119" s="24" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C119" s="24" t="inlineStr">
@@ -19272,7 +19272,7 @@
       </c>
       <c r="E119" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; is cancelled" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "PDC warehouse updated" (type Confirmation).</t>
         </is>
       </c>
       <c r="F119" s="24" t="inlineStr">
@@ -19305,12 +19305,12 @@
     <row r="120">
       <c r="A120" s="22" t="inlineStr">
         <is>
-          <t>M-118</t>
+          <t>M-148</t>
         </is>
       </c>
       <c r="B120" s="22" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C120" s="22" t="inlineStr">
@@ -19325,7 +19325,7 @@
       </c>
       <c r="E120" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt; has no failures" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A post-dated check needs an amount above zero" (type Error).</t>
         </is>
       </c>
       <c r="F120" s="22" t="inlineStr">
@@ -19358,12 +19358,12 @@
     <row r="121">
       <c r="A121" s="24" t="inlineStr">
         <is>
-          <t>M-119</t>
+          <t>M-149</t>
         </is>
       </c>
       <c r="B121" s="24" t="inlineStr">
         <is>
-          <t>Batch Print (SCR-OP-18)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C121" s="24" t="inlineStr">
@@ -19378,7 +19378,7 @@
       </c>
       <c r="E121" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Select between 1 and 500 receipts to print" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Check &lt;bank code&gt; &lt;check no&gt; is already warehoused" (type Error).</t>
         </is>
       </c>
       <c r="F121" s="24" t="inlineStr">
@@ -19411,12 +19411,12 @@
     <row r="122">
       <c r="A122" s="22" t="inlineStr">
         <is>
-          <t>M-140</t>
+          <t>M-150</t>
         </is>
       </c>
       <c r="B122" s="22" t="inlineStr">
         <is>
-          <t>Commission ORs (SCR-OP-20)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C122" s="22" t="inlineStr">
@@ -19431,7 +19431,7 @@
       </c>
       <c r="E122" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No commission payment waiting for an OR" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Check &lt;warehouse no&gt; is &lt;status&gt;, not in the warehouse" (type Error).</t>
         </is>
       </c>
       <c r="F122" s="22" t="inlineStr">
@@ -19464,12 +19464,12 @@
     <row r="123">
       <c r="A123" s="24" t="inlineStr">
         <is>
-          <t>M-141</t>
+          <t>M-151</t>
         </is>
       </c>
       <c r="B123" s="24" t="inlineStr">
         <is>
-          <t>Commission ORs (SCR-OP-20)</t>
+          <t>PDC Warehouse (SCR-OP-16)</t>
         </is>
       </c>
       <c r="C123" s="24" t="inlineStr">
@@ -19484,7 +19484,7 @@
       </c>
       <c r="E123" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown company &lt;company&gt;" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "A check leaves the warehouse as returned, replaced or pulled out" (type Error).</t>
         </is>
       </c>
       <c r="F123" s="24" t="inlineStr">
@@ -19517,12 +19517,12 @@
     <row r="124">
       <c r="A124" s="22" t="inlineStr">
         <is>
-          <t>M-351</t>
+          <t>M-152</t>
         </is>
       </c>
       <c r="B124" s="22" t="inlineStr">
         <is>
-          <t>Interfaces (SCR-OP-61)</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C124" s="22" t="inlineStr">
@@ -19537,7 +19537,7 @@
       </c>
       <c r="E124" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;name&gt; saved" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt;: &lt;printed count&gt; printed, &lt;failed count&gt; not printed" (type Confirmation).</t>
         </is>
       </c>
       <c r="F124" s="22" t="inlineStr">
@@ -19570,12 +19570,12 @@
     <row r="125">
       <c r="A125" s="24" t="inlineStr">
         <is>
-          <t>M-352</t>
+          <t>M-153</t>
         </is>
       </c>
       <c r="B125" s="24" t="inlineStr">
         <is>
-          <t>Interfaces (SCR-OP-61)</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C125" s="24" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="E125" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No records in this run" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Receipt &lt;receipt no&gt; is cancelled" (type Error).</t>
         </is>
       </c>
       <c r="F125" s="24" t="inlineStr">
@@ -19623,12 +19623,12 @@
     <row r="126">
       <c r="A126" s="22" t="inlineStr">
         <is>
-          <t>M-353</t>
+          <t>M-154</t>
         </is>
       </c>
       <c r="B126" s="22" t="inlineStr">
         <is>
-          <t>Interfaces (SCR-OP-61)</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C126" s="22" t="inlineStr">
@@ -19643,7 +19643,7 @@
       </c>
       <c r="E126" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No runs yet" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt; has no failure to skip" (type Error).</t>
         </is>
       </c>
       <c r="F126" s="22" t="inlineStr">
@@ -19676,12 +19676,12 @@
     <row r="127">
       <c r="A127" s="24" t="inlineStr">
         <is>
-          <t>M-354</t>
+          <t>M-155</t>
         </is>
       </c>
       <c r="B127" s="24" t="inlineStr">
         <is>
-          <t>Interfaces (SCR-OP-61)</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C127" s="24" t="inlineStr">
@@ -19696,7 +19696,7 @@
       </c>
       <c r="E127" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Feed &lt;code&gt; is inactive" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt; has no failures" (type Error).</t>
         </is>
       </c>
       <c r="F127" s="24" t="inlineStr">
@@ -19729,12 +19729,12 @@
     <row r="128">
       <c r="A128" s="22" t="inlineStr">
         <is>
-          <t>M-355</t>
+          <t>M-156</t>
         </is>
       </c>
       <c r="B128" s="22" t="inlineStr">
         <is>
-          <t>Interfaces (SCR-OP-61)</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C128" s="22" t="inlineStr">
@@ -19749,7 +19749,7 @@
       </c>
       <c r="E128" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No module processes uploads of feed &lt;feed code&gt; yet" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;batch no&gt; has no ZIP of its receipts" (type Error).</t>
         </is>
       </c>
       <c r="F128" s="22" t="inlineStr">
@@ -19782,12 +19782,12 @@
     <row r="129">
       <c r="A129" s="24" t="inlineStr">
         <is>
-          <t>M-356</t>
+          <t>M-157</t>
         </is>
       </c>
       <c r="B129" s="24" t="inlineStr">
         <is>
-          <t>Several screens</t>
+          <t>Batch Print (SCR-OP-18)</t>
         </is>
       </c>
       <c r="C129" s="24" t="inlineStr">
@@ -19802,7 +19802,7 @@
       </c>
       <c r="E129" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "No receipt series yet" (type Information).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Select between 1 and 500 receipts to print" (type Error).</t>
         </is>
       </c>
       <c r="F129" s="24" t="inlineStr">
@@ -19835,12 +19835,12 @@
     <row r="130">
       <c r="A130" s="22" t="inlineStr">
         <is>
-          <t>M-357</t>
+          <t>M-178</t>
         </is>
       </c>
       <c r="B130" s="22" t="inlineStr">
         <is>
-          <t>Several screens</t>
+          <t>Commission ORs (SCR-OP-20)</t>
         </is>
       </c>
       <c r="C130" s="22" t="inlineStr">
@@ -19855,7 +19855,7 @@
       </c>
       <c r="E130" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Prefix is required" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No commission payment waiting for an OR" (type Information).</t>
         </is>
       </c>
       <c r="F130" s="22" t="inlineStr">
@@ -19888,12 +19888,12 @@
     <row r="131">
       <c r="A131" s="24" t="inlineStr">
         <is>
-          <t>M-358</t>
+          <t>M-179</t>
         </is>
       </c>
       <c r="B131" s="24" t="inlineStr">
         <is>
-          <t>Several screens</t>
+          <t>Commission ORs (SCR-OP-20)</t>
         </is>
       </c>
       <c r="C131" s="24" t="inlineStr">
@@ -19908,7 +19908,7 @@
       </c>
       <c r="E131" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Series &lt;prefix&gt; saved" (type Confirmation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Unknown company &lt;company&gt;" (type Error).</t>
         </is>
       </c>
       <c r="F131" s="24" t="inlineStr">
@@ -19941,12 +19941,12 @@
     <row r="132">
       <c r="A132" s="22" t="inlineStr">
         <is>
-          <t>M-359</t>
+          <t>M-389</t>
         </is>
       </c>
       <c r="B132" s="22" t="inlineStr">
         <is>
-          <t>Several screens</t>
+          <t>Interfaces (SCR-OP-61)</t>
         </is>
       </c>
       <c r="C132" s="22" t="inlineStr">
@@ -19961,7 +19961,7 @@
       </c>
       <c r="E132" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The range must end at or after its start" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;name&gt; saved" (type Confirmation).</t>
         </is>
       </c>
       <c r="F132" s="22" t="inlineStr">
@@ -19994,12 +19994,12 @@
     <row r="133">
       <c r="A133" s="24" t="inlineStr">
         <is>
-          <t>M-360</t>
+          <t>M-390</t>
         </is>
       </c>
       <c r="B133" s="24" t="inlineStr">
         <is>
-          <t>Several screens</t>
+          <t>Interfaces (SCR-OP-61)</t>
         </is>
       </c>
       <c r="C133" s="24" t="inlineStr">
@@ -20014,7 +20014,7 @@
       </c>
       <c r="E133" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The series becomes active for issuing receipts." (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No records in this run" (type Information).</t>
         </is>
       </c>
       <c r="F133" s="24" t="inlineStr">
@@ -20047,12 +20047,12 @@
     <row r="134">
       <c r="A134" s="22" t="inlineStr">
         <is>
-          <t>M-361</t>
+          <t>M-391</t>
         </is>
       </c>
       <c r="B134" s="22" t="inlineStr">
         <is>
-          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+          <t>Interfaces (SCR-OP-61)</t>
         </is>
       </c>
       <c r="C134" s="22" t="inlineStr">
@@ -20067,7 +20067,7 @@
       </c>
       <c r="E134" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No runs yet" (type Information).</t>
         </is>
       </c>
       <c r="F134" s="22" t="inlineStr">
@@ -20100,12 +20100,12 @@
     <row r="135">
       <c r="A135" s="24" t="inlineStr">
         <is>
-          <t>M-362</t>
+          <t>M-392</t>
         </is>
       </c>
       <c r="B135" s="24" t="inlineStr">
         <is>
-          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+          <t>Interfaces (SCR-OP-61)</t>
         </is>
       </c>
       <c r="C135" s="24" t="inlineStr">
@@ -20120,7 +20120,7 @@
       </c>
       <c r="E135" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;Column&gt; is mandatory" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Feed &lt;code&gt; is inactive" (type Error).</t>
         </is>
       </c>
       <c r="F135" s="24" t="inlineStr">
@@ -20153,12 +20153,12 @@
     <row r="136">
       <c r="A136" s="22" t="inlineStr">
         <is>
-          <t>M-366</t>
+          <t>M-393</t>
         </is>
       </c>
       <c r="B136" s="22" t="inlineStr">
         <is>
-          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+          <t>Interfaces (SCR-OP-61)</t>
         </is>
       </c>
       <c r="C136" s="22" t="inlineStr">
@@ -20173,7 +20173,7 @@
       </c>
       <c r="E136" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The amount must be above zero" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No module processes uploads of feed &lt;feed code&gt; yet" (type Error).</t>
         </is>
       </c>
       <c r="F136" s="22" t="inlineStr">
@@ -20206,12 +20206,12 @@
     <row r="137">
       <c r="A137" s="24" t="inlineStr">
         <is>
-          <t>M-367</t>
+          <t>M-394</t>
         </is>
       </c>
       <c r="B137" s="24" t="inlineStr">
         <is>
-          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C137" s="24" t="inlineStr">
@@ -20226,7 +20226,7 @@
       </c>
       <c r="E137" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The basic commission must be above zero" (type Validation).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "No receipt series yet" (type Information).</t>
         </is>
       </c>
       <c r="F137" s="24" t="inlineStr">
@@ -20259,12 +20259,12 @@
     <row r="138">
       <c r="A138" s="22" t="inlineStr">
         <is>
-          <t>M-368</t>
+          <t>M-395</t>
         </is>
       </c>
       <c r="B138" s="22" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C138" s="22" t="inlineStr">
@@ -20279,7 +20279,7 @@
       </c>
       <c r="E138" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "You are not permitted to perform this action" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Nothing to show" (type Information).</t>
         </is>
       </c>
       <c r="F138" s="22" t="inlineStr">
@@ -20312,12 +20312,12 @@
     <row r="139">
       <c r="A139" s="24" t="inlineStr">
         <is>
-          <t>M-369</t>
+          <t>M-396</t>
         </is>
       </c>
       <c r="B139" s="24" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C139" s="24" t="inlineStr">
@@ -20332,7 +20332,7 @@
       </c>
       <c r="E139" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The record was changed by another user. Please reload and try again." (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Prefix is required" (type Validation).</t>
         </is>
       </c>
       <c r="F139" s="24" t="inlineStr">
@@ -20365,12 +20365,12 @@
     <row r="140">
       <c r="A140" s="22" t="inlineStr">
         <is>
-          <t>M-370</t>
+          <t>M-397</t>
         </is>
       </c>
       <c r="B140" s="22" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C140" s="22" t="inlineStr">
@@ -20385,7 +20385,7 @@
       </c>
       <c r="E140" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The system could not complete the request. Try again; if it continues, contact support with the reference." (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Series &lt;prefix&gt; saved" (type Confirmation).</t>
         </is>
       </c>
       <c r="F140" s="22" t="inlineStr">
@@ -20418,12 +20418,12 @@
     <row r="141">
       <c r="A141" s="24" t="inlineStr">
         <is>
-          <t>M-371</t>
+          <t>M-398</t>
         </is>
       </c>
       <c r="B141" s="24" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C141" s="24" t="inlineStr">
@@ -20438,7 +20438,7 @@
       </c>
       <c r="E141" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Parameter '&lt;name&gt;' has an invalid value" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The number format must hold the sequence {SEQ}" (type Validation).</t>
         </is>
       </c>
       <c r="F141" s="24" t="inlineStr">
@@ -20471,12 +20471,12 @@
     <row r="142">
       <c r="A142" s="22" t="inlineStr">
         <is>
-          <t>M-372</t>
+          <t>M-399</t>
         </is>
       </c>
       <c r="B142" s="22" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C142" s="22" t="inlineStr">
@@ -20491,7 +20491,7 @@
       </c>
       <c r="E142" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Required parameter '&lt;parameter name&gt;' is missing" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The range must end at or after its start" (type Validation).</t>
         </is>
       </c>
       <c r="F142" s="22" t="inlineStr">
@@ -20524,12 +20524,12 @@
     <row r="143">
       <c r="A143" s="24" t="inlineStr">
         <is>
-          <t>M-373</t>
+          <t>M-400</t>
         </is>
       </c>
       <c r="B143" s="24" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Several screens</t>
         </is>
       </c>
       <c r="C143" s="24" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="E143" s="24" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "The uploaded file is too large" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The series becomes active for issuing receipts." (type Validation).</t>
         </is>
       </c>
       <c r="F143" s="24" t="inlineStr">
@@ -20577,12 +20577,12 @@
     <row r="144">
       <c r="A144" s="22" t="inlineStr">
         <is>
-          <t>M-374</t>
+          <t>M-401</t>
         </is>
       </c>
       <c r="B144" s="22" t="inlineStr">
         <is>
-          <t>Every screen (Common screen elements)</t>
+          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
         </is>
       </c>
       <c r="C144" s="22" t="inlineStr">
@@ -20597,7 +20597,7 @@
       </c>
       <c r="E144" s="22" t="inlineStr">
         <is>
-          <t>Confirm the wording of the message, or give BDOI's wording: "Invalid request" (type Error).</t>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;" (type Validation).</t>
         </is>
       </c>
       <c r="F144" s="22" t="inlineStr">
@@ -20627,8 +20627,962 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="24" t="inlineStr">
+        <is>
+          <t>M-402</t>
+        </is>
+      </c>
+      <c r="B145" s="24" t="inlineStr">
+        <is>
+          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+        </is>
+      </c>
+      <c r="C145" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D145" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E145" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;Column&gt; is mandatory" (type Validation).</t>
+        </is>
+      </c>
+      <c r="F145" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G145" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H145" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I145" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J145" s="24" t="inlineStr"/>
+      <c r="K145" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="22" t="inlineStr">
+        <is>
+          <t>M-406</t>
+        </is>
+      </c>
+      <c r="B146" s="22" t="inlineStr">
+        <is>
+          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+        </is>
+      </c>
+      <c r="C146" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D146" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E146" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The amount must be above zero" (type Validation).</t>
+        </is>
+      </c>
+      <c r="F146" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G146" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H146" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I146" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J146" s="22" t="inlineStr"/>
+      <c r="K146" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="24" t="inlineStr">
+        <is>
+          <t>M-407</t>
+        </is>
+      </c>
+      <c r="B147" s="24" t="inlineStr">
+        <is>
+          <t>Upload screens (Payment Uploads, BIR 2307, Commission ORs, B</t>
+        </is>
+      </c>
+      <c r="C147" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D147" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E147" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The basic commission must be above zero" (type Validation).</t>
+        </is>
+      </c>
+      <c r="F147" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G147" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H147" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I147" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J147" s="24" t="inlineStr"/>
+      <c r="K147" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="22" t="inlineStr">
+        <is>
+          <t>M-408</t>
+        </is>
+      </c>
+      <c r="B148" s="22" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C148" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D148" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E148" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "You are not permitted to perform this action" (type Error).</t>
+        </is>
+      </c>
+      <c r="F148" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G148" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H148" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I148" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J148" s="22" t="inlineStr"/>
+      <c r="K148" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="24" t="inlineStr">
+        <is>
+          <t>M-409</t>
+        </is>
+      </c>
+      <c r="B149" s="24" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C149" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D149" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E149" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Enter the code and the name" (type Error).</t>
+        </is>
+      </c>
+      <c r="F149" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G149" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H149" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I149" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J149" s="24" t="inlineStr"/>
+      <c r="K149" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="22" t="inlineStr">
+        <is>
+          <t>M-410</t>
+        </is>
+      </c>
+      <c r="B150" s="22" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C150" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D150" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E150" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Write each field as Field=position or Field=column, not '&lt;part&gt;'" (type Error).</t>
+        </is>
+      </c>
+      <c r="F150" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G150" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H150" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I150" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J150" s="22" t="inlineStr"/>
+      <c r="K150" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="24" t="inlineStr">
+        <is>
+          <t>M-411</t>
+        </is>
+      </c>
+      <c r="B151" s="24" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C151" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D151" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E151" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The file cannot be read as an Excel workbook" (type Error).</t>
+        </is>
+      </c>
+      <c r="F151" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G151" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H151" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I151" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J151" s="24" t="inlineStr"/>
+      <c r="K151" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="22" t="inlineStr">
+        <is>
+          <t>M-412</t>
+        </is>
+      </c>
+      <c r="B152" s="22" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C152" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D152" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E152" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The file name convention is not a valid pattern" (type Error).</t>
+        </is>
+      </c>
+      <c r="F152" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G152" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H152" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I152" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J152" s="22" t="inlineStr"/>
+      <c r="K152" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="24" t="inlineStr">
+        <is>
+          <t>M-413</t>
+        </is>
+      </c>
+      <c r="B153" s="24" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C153" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D153" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E153" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The record was changed by another user. Please reload and try again." (type Error).</t>
+        </is>
+      </c>
+      <c r="F153" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G153" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H153" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I153" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J153" s="24" t="inlineStr"/>
+      <c r="K153" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="22" t="inlineStr">
+        <is>
+          <t>M-414</t>
+        </is>
+      </c>
+      <c r="B154" s="22" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C154" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D154" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E154" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Version &lt;version no&gt; is not waiting for approval" (type Error).</t>
+        </is>
+      </c>
+      <c r="F154" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G154" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H154" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I154" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J154" s="22" t="inlineStr"/>
+      <c r="K154" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="24" t="inlineStr">
+        <is>
+          <t>M-415</t>
+        </is>
+      </c>
+      <c r="B155" s="24" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C155" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D155" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E155" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The system could not complete the request. Try again; if it continues, contact support with the reference." (type Error).</t>
+        </is>
+      </c>
+      <c r="F155" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G155" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H155" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I155" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J155" s="24" t="inlineStr"/>
+      <c r="K155" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="22" t="inlineStr">
+        <is>
+          <t>M-416</t>
+        </is>
+      </c>
+      <c r="B156" s="22" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C156" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D156" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E156" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The user who changed the form cannot approve it" (type Error).</t>
+        </is>
+      </c>
+      <c r="F156" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G156" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H156" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I156" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J156" s="22" t="inlineStr"/>
+      <c r="K156" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="24" t="inlineStr">
+        <is>
+          <t>M-417</t>
+        </is>
+      </c>
+      <c r="B157" s="24" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C157" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D157" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E157" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Parameter '&lt;name&gt;' has an invalid value" (type Error).</t>
+        </is>
+      </c>
+      <c r="F157" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G157" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H157" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I157" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J157" s="24" t="inlineStr"/>
+      <c r="K157" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="22" t="inlineStr">
+        <is>
+          <t>M-418</t>
+        </is>
+      </c>
+      <c r="B158" s="22" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C158" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D158" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E158" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Required parameter '&lt;parameter name&gt;' is missing" (type Error).</t>
+        </is>
+      </c>
+      <c r="F158" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G158" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H158" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I158" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J158" s="22" t="inlineStr"/>
+      <c r="K158" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="24" t="inlineStr">
+        <is>
+          <t>M-419</t>
+        </is>
+      </c>
+      <c r="B159" s="24" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C159" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D159" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E159" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "&lt;name&gt; has no MFT folder" (type Error).</t>
+        </is>
+      </c>
+      <c r="F159" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G159" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H159" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I159" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J159" s="24" t="inlineStr"/>
+      <c r="K159" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="22" t="inlineStr">
+        <is>
+          <t>M-420</t>
+        </is>
+      </c>
+      <c r="B160" s="22" t="inlineStr">
+        <is>
+          <t>Several screens</t>
+        </is>
+      </c>
+      <c r="C160" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D160" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E160" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "An &lt;kind&gt; is issued when its creation record is posted: save it with Create &lt;kind&gt; and submit it for posting" (type Error).</t>
+        </is>
+      </c>
+      <c r="F160" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G160" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H160" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I160" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J160" s="22" t="inlineStr"/>
+      <c r="K160" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="24" t="inlineStr">
+        <is>
+          <t>M-421</t>
+        </is>
+      </c>
+      <c r="B161" s="24" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C161" s="24" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D161" s="24" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E161" s="24" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "The uploaded file is too large" (type Error).</t>
+        </is>
+      </c>
+      <c r="F161" s="24" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G161" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H161" s="24" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I161" s="24" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J161" s="24" t="inlineStr"/>
+      <c r="K161" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="22" t="inlineStr">
+        <is>
+          <t>M-422</t>
+        </is>
+      </c>
+      <c r="B162" s="22" t="inlineStr">
+        <is>
+          <t>Every screen (Common screen elements)</t>
+        </is>
+      </c>
+      <c r="C162" s="22" t="inlineStr">
+        <is>
+          <t>CSHID.001-025</t>
+        </is>
+      </c>
+      <c r="D162" s="22" t="inlineStr">
+        <is>
+          <t>Appendix F.2</t>
+        </is>
+      </c>
+      <c r="E162" s="22" t="inlineStr">
+        <is>
+          <t>Confirm the wording of the message, or give BDOI's wording: "Invalid request" (type Error).</t>
+        </is>
+      </c>
+      <c r="F162" s="22" t="inlineStr">
+        <is>
+          <t>Confirm, or the new wording</t>
+        </is>
+      </c>
+      <c r="G162" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H162" s="22" t="inlineStr">
+        <is>
+          <t>Cashiering Process Owner</t>
+        </is>
+      </c>
+      <c r="I162" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J162" s="22" t="inlineStr"/>
+      <c r="K162" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A12:K144"/>
+  <autoFilter ref="A12:K162"/>
   <mergeCells count="5">
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="B6:K6"/>
@@ -20637,7 +21591,7 @@
     <mergeCell ref="B5:K5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K14:K444" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="K14:K462" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>